<commit_message>
Add EC2 deployment scripts for 20 parallel servers
- ec2-userdata.sh: Ubuntu user data (Node, Playwright, Xvfb setup)
- deploy-ec2.sh: AWS CLI to launch 20 instances at once
- distribute-session.sh: Push local session.json to all servers
- trigger-all.sh: Start tests on all servers simultaneously
- Enable parallel execution with 20 workers in playwright config
- Update session.json with fresh auth cookies

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/applications/applications.xlsx
+++ b/data/applications/applications.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GCV\Rayna Automation\data\applications\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E9B0CEB-93D3-40D9-8050-78BF354D060B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2C9246F-C4DC-417F-B2DA-937D1BE88211}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="83">
   <si>
     <t>Full Name</t>
   </si>
@@ -645,8 +645,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AV2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AV3"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -697,7 +697,7 @@
     <col min="48" max="48" width="23.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:48" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -843,7 +843,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:48" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:48" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -986,6 +986,152 @@
         <v>80</v>
       </c>
       <c r="AV2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:48" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" t="s">
+        <v>54</v>
+      </c>
+      <c r="I3" t="s">
+        <v>55</v>
+      </c>
+      <c r="J3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" t="s">
+        <v>55</v>
+      </c>
+      <c r="L3" t="s">
+        <v>56</v>
+      </c>
+      <c r="M3" t="s">
+        <v>55</v>
+      </c>
+      <c r="N3" t="s">
+        <v>57</v>
+      </c>
+      <c r="O3" t="s">
+        <v>58</v>
+      </c>
+      <c r="P3" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>59</v>
+      </c>
+      <c r="R3" t="s">
+        <v>60</v>
+      </c>
+      <c r="S3" t="s">
+        <v>61</v>
+      </c>
+      <c r="T3" t="s">
+        <v>62</v>
+      </c>
+      <c r="U3" t="s">
+        <v>63</v>
+      </c>
+      <c r="V3" t="s">
+        <v>64</v>
+      </c>
+      <c r="W3" t="s">
+        <v>65</v>
+      </c>
+      <c r="X3" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>66</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>68</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>69</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>70</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>71</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>72</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>73</v>
+      </c>
+      <c r="AM3" t="s">
+        <v>74</v>
+      </c>
+      <c r="AN3" t="s">
+        <v>75</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>76</v>
+      </c>
+      <c r="AP3" t="s">
+        <v>77</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>78</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT3" t="s">
+        <v>79</v>
+      </c>
+      <c r="AU3" t="s">
+        <v>80</v>
+      </c>
+      <c r="AV3" t="s">
         <v>81</v>
       </c>
     </row>

</xml_diff>